<commit_message>
feat: Add custom refill modes, EDT & Elixir ratios, own bottle, Mayar & Biteship integrations
</commit_message>
<xml_diff>
--- a/public/assets/Data Bibit Botol Ela parfum.xlsx
+++ b/public/assets/Data Bibit Botol Ela parfum.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Abu Bakar Al Adny\OneDrive\Dokumen\Project Web\Minyak Wangi\public\assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5de607373dc178dc/Dokumen/Project Web/Minyak Wangi/public/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C966180-9255-4559-AC6D-7ACEA4E26AD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{7C966180-9255-4559-AC6D-7ACEA4E26AD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC4F2AAA-0BF7-4D87-9382-75034176751E}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A1658247-E350-4980-A13D-CC21F9607D75}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{A1658247-E350-4980-A13D-CC21F9607D75}"/>
   </bookViews>
   <sheets>
     <sheet name="Parfum Umum" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1557" uniqueCount="1485">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1536" uniqueCount="1484">
   <si>
     <t>NO</t>
   </si>
@@ -19215,9 +19215,6 @@
   </si>
   <si>
     <t>CASA 50ML</t>
-  </si>
-  <si>
-    <t>JO MALONE 50ML</t>
   </si>
   <si>
     <t>XX/POT 50ML</t>
@@ -27983,7 +27980,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D33D2B56-140A-4CE8-B536-8A2963B19C42}">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
@@ -28000,99 +27997,106 @@
         <v>1451</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>1472</v>
+        <v>1471</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>1452</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
-        <v>3</v>
+      <c r="A2" s="3">
+        <f>1</f>
+        <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>1453</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>1477</v>
+        <v>1476</v>
       </c>
       <c r="D2" s="5">
         <v>10000</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>5</v>
+      <c r="A3" s="3">
+        <f>A2+1</f>
+        <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>1454</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>1473</v>
+        <v>1472</v>
       </c>
       <c r="D3" s="5">
         <v>10000</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>7</v>
+      <c r="A4" s="3">
+        <f t="shared" ref="A4:A19" si="0">A3+1</f>
+        <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>1455</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>1473</v>
+        <v>1472</v>
       </c>
       <c r="D4" s="5">
         <v>10000</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>9</v>
+      <c r="A5" s="3">
+        <f t="shared" si="0"/>
+        <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>1456</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>1473</v>
+        <v>1472</v>
       </c>
       <c r="D5" s="5">
         <v>10000</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>11</v>
+      <c r="A6" s="3">
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>1457</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>1474</v>
+        <v>1473</v>
       </c>
       <c r="D6" s="5">
         <v>10000</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>13</v>
+      <c r="A7" s="3">
+        <f t="shared" si="0"/>
+        <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>1458</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>1474</v>
+        <v>1473</v>
       </c>
       <c r="D7" s="5">
         <v>10000</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>15</v>
+      <c r="A8" s="3">
+        <f t="shared" si="0"/>
+        <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>1459</v>
@@ -28105,8 +28109,9 @@
       </c>
     </row>
     <row r="9" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
-        <v>17</v>
+      <c r="A9" s="3">
+        <f t="shared" si="0"/>
+        <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>1460</v>
@@ -28119,8 +28124,9 @@
       </c>
     </row>
     <row r="10" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>19</v>
+      <c r="A10" s="3">
+        <f t="shared" si="0"/>
+        <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>1461</v>
@@ -28129,12 +28135,13 @@
         <v>1476</v>
       </c>
       <c r="D10" s="5">
-        <v>10000</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
-        <v>21</v>
+      <c r="A11" s="3">
+        <f t="shared" si="0"/>
+        <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>1462</v>
@@ -28147,8 +28154,9 @@
       </c>
     </row>
     <row r="12" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="3" t="s">
-        <v>23</v>
+      <c r="A12" s="3">
+        <f t="shared" si="0"/>
+        <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>1463</v>
@@ -28161,22 +28169,24 @@
       </c>
     </row>
     <row r="13" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
-        <v>25</v>
+      <c r="A13" s="3">
+        <f t="shared" si="0"/>
+        <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>1464</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>1479</v>
+        <v>1474</v>
       </c>
       <c r="D13" s="5">
-        <v>2500</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="3" t="s">
-        <v>27</v>
+      <c r="A14" s="3">
+        <f t="shared" si="0"/>
+        <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>1465</v>
@@ -28189,22 +28199,24 @@
       </c>
     </row>
     <row r="15" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="3" t="s">
-        <v>29</v>
+      <c r="A15" s="3">
+        <f t="shared" si="0"/>
+        <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>1466</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>1476</v>
+        <v>1479</v>
       </c>
       <c r="D15" s="5">
-        <v>3000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="3" t="s">
-        <v>31</v>
+      <c r="A16" s="3">
+        <f t="shared" si="0"/>
+        <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>1467</v>
@@ -28217,8 +28229,9 @@
       </c>
     </row>
     <row r="17" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="3" t="s">
-        <v>33</v>
+      <c r="A17" s="3">
+        <f t="shared" si="0"/>
+        <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>1468</v>
@@ -28231,8 +28244,9 @@
       </c>
     </row>
     <row r="18" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="3" t="s">
-        <v>35</v>
+      <c r="A18" s="3">
+        <f t="shared" si="0"/>
+        <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>1469</v>
@@ -28241,12 +28255,13 @@
         <v>1482</v>
       </c>
       <c r="D18" s="5">
-        <v>2000</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="3" t="s">
-        <v>37</v>
+      <c r="A19" s="3">
+        <f t="shared" si="0"/>
+        <v>18</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>1470</v>
@@ -28255,20 +28270,6 @@
         <v>1483</v>
       </c>
       <c r="D19" s="5">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>1471</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>1484</v>
-      </c>
-      <c r="D20" s="5">
         <v>2500</v>
       </c>
     </row>

</xml_diff>